<commit_message>
Initial debugging after merge
</commit_message>
<xml_diff>
--- a/Utilities/titles/VariableListing.xlsx
+++ b/Utilities/titles/VariableListing.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Work profile\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Work profile\Documents\GitHub\FTT_StandAlone\Utilities\titles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6FBE3B-9D55-418B-9038-FD51099BA3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820AC22B-2FED-4142-995A-27D7F6AF9D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10305" windowHeight="17400" xr2:uid="{3966A5EA-18B5-40FC-82B6-8DC341B5B05B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{3966A5EA-18B5-40FC-82B6-8DC341B5B05B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3421,7 +3421,7 @@
         <v>9</v>
       </c>
       <c r="K14">
-        <v>2001</v>
+        <v>2010</v>
       </c>
       <c r="L14" t="s">
         <v>9</v>
@@ -6085,7 +6085,7 @@
         <v>9</v>
       </c>
       <c r="K81">
-        <v>2001</v>
+        <v>2010</v>
       </c>
       <c r="L81" t="s">
         <v>9</v>

</xml_diff>